<commit_message>
Validated Net housing wealth
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyFiles\99 DEV ENV\JAS-MINE\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B4A97A-11EB-43BF-9DFE-4390FC3D442C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F39765-0403-4026-9E5B-556F09754A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4620" yWindow="1750" windowWidth="28800" windowHeight="15290" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -118,6 +129,12 @@
   </si>
   <si>
     <t>FW1a</t>
+  </si>
+  <si>
+    <t>HW1c</t>
+  </si>
+  <si>
+    <t>HW1d</t>
   </si>
 </sst>
 </file>
@@ -486,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38.1796875" customWidth="1"/>
@@ -732,6 +749,22 @@
         <v>0.50560000000000005</v>
       </c>
     </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
+        <v>0.95802536417754225</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>2.3250999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct unsecured-debt covariates and persistence estimates
- Jointly estimate annual persistence and coefficients for the continuing low- and high-cost debt equations, exporting their full covariance matrices and updated RMSEs.
- Added PrivateIncomeQuintile2-5 by collapsing the existing private-income deciles. Previously the models ran successfully but used Java’s unrelated model-wide income quintiles.
- Update the FW2a clustered covariance matrix.
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UK" sheetId="1" r:id="R79d909dd203b4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UK" sheetId="1" r:id="R52cca3e2589e4f37"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -85,9 +85,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -479,7 +479,7 @@
         <x:v>FW2c</x:v>
       </x:c>
       <x:c r="B36" t="n">
-        <x:v>1.1064186435860763</x:v>
+        <x:v>1.13574141020715</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -495,7 +495,7 @@
         <x:v>FW2e</x:v>
       </x:c>
       <x:c r="B38" t="n">
-        <x:v>1.004758156254813</x:v>
+        <x:v>0.9720760974457268</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>